<commit_message>
feature: tự động tạo classSubject
</commit_message>
<xml_diff>
--- a/src/assets/bangdiem_template.xlsx
+++ b/src/assets/bangdiem_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace\QuanTriTruongHoc_BE\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CCE4A5D-F357-42DB-B396-92EFFACC2F0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21EBFD5C-00F7-4AE2-9340-F4844731D463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5E6F906E-4952-4227-9D02-B0001F3530D5}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
   <si>
     <t xml:space="preserve">KẾT QUẢ HỌC TẬP MÔN HỌC/MÔ ĐUN
 TIN HỌC VĂN PHÒNG        </t>
@@ -73,7 +73,37 @@
     <t>Họ tên</t>
   </si>
   <si>
-    <t>{{gradeColumns}}</t>
+    <t>KTTX</t>
+  </si>
+  <si>
+    <t>Lần 1</t>
+  </si>
+  <si>
+    <t>Lần 2</t>
+  </si>
+  <si>
+    <t>Lần 3</t>
+  </si>
+  <si>
+    <t>Kiểm tra định kỳ</t>
+  </si>
+  <si>
+    <t>Lần 4</t>
+  </si>
+  <si>
+    <t>Trung bình</t>
+  </si>
+  <si>
+    <t>Điểm kiểm tra</t>
+  </si>
+  <si>
+    <t>Tổng kết lần 1</t>
+  </si>
+  <si>
+    <t>Tổng kết lần 2</t>
+  </si>
+  <si>
+    <t>Ghi chú</t>
   </si>
 </sst>
 </file>
@@ -143,7 +173,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -151,11 +181,99 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -167,6 +285,48 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -179,47 +339,38 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -535,36 +686,38 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{126F2789-0FE7-4317-A3A6-DB05700D32CA}">
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="21.44140625" customWidth="1"/>
     <col min="4" max="4" width="16.44140625" customWidth="1"/>
-    <col min="5" max="5" width="25.44140625" customWidth="1"/>
-    <col min="6" max="6" width="14.77734375" customWidth="1"/>
-    <col min="7" max="7" width="17.5546875" customWidth="1"/>
-    <col min="8" max="8" width="14.6640625" customWidth="1"/>
-    <col min="10" max="10" width="13.88671875" customWidth="1"/>
+    <col min="5" max="5" width="9.6640625" customWidth="1"/>
+    <col min="6" max="7" width="8.21875" customWidth="1"/>
+    <col min="8" max="8" width="8.109375" customWidth="1"/>
+    <col min="10" max="10" width="8.77734375" customWidth="1"/>
+    <col min="12" max="12" width="12.33203125" customWidth="1"/>
+    <col min="15" max="15" width="15.109375" customWidth="1"/>
+    <col min="16" max="16" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-    </row>
-    <row r="2" spans="1:13" ht="18" x14ac:dyDescent="0.3">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+    </row>
+    <row r="2" spans="1:17" ht="18" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
@@ -583,7 +736,7 @@
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
     </row>
-    <row r="3" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
@@ -602,7 +755,7 @@
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
     </row>
-    <row r="4" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
@@ -621,7 +774,7 @@
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
     </row>
-    <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="1"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -636,360 +789,398 @@
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
     </row>
-    <row r="6" spans="1:13" ht="54" x14ac:dyDescent="0.3">
-      <c r="A6" s="9" t="s">
+    <row r="6" spans="1:17" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-    </row>
-    <row r="7" spans="1:13" ht="18" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-    </row>
-    <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.3">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-    </row>
-    <row r="9" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A9" s="11"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="15"/>
-      <c r="K9" s="15"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
-    </row>
-    <row r="10" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A10" s="11"/>
-      <c r="B10" s="18"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="15"/>
-      <c r="K10" s="15"/>
-      <c r="L10" s="17"/>
-      <c r="M10" s="17"/>
-    </row>
-    <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A11" s="11"/>
-      <c r="B11" s="18"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="16"/>
-      <c r="J11" s="15"/>
-      <c r="K11" s="15"/>
-      <c r="L11" s="17"/>
-      <c r="M11" s="17"/>
-    </row>
-    <row r="12" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A12" s="11"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="15"/>
-      <c r="K12" s="15"/>
-      <c r="L12" s="17"/>
-      <c r="M12" s="17"/>
-    </row>
-    <row r="13" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A13" s="11"/>
-      <c r="B13" s="19"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="16"/>
-      <c r="J13" s="15"/>
-      <c r="K13" s="15"/>
-      <c r="L13" s="17"/>
-      <c r="M13" s="17"/>
-    </row>
-    <row r="14" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A14" s="11"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="16"/>
-      <c r="J14" s="15"/>
-      <c r="K14" s="15"/>
-      <c r="L14" s="17"/>
-      <c r="M14" s="17"/>
-    </row>
-    <row r="15" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A15" s="11"/>
-      <c r="B15" s="19"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="15"/>
-      <c r="L15" s="17"/>
-      <c r="M15" s="17"/>
-    </row>
-    <row r="16" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A16" s="11"/>
-      <c r="B16" s="21"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="16"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="15"/>
-      <c r="L16" s="17"/>
-      <c r="M16" s="17"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="I6" s="30"/>
+      <c r="J6" s="30"/>
+      <c r="K6" s="31"/>
+      <c r="L6" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="M6" s="29" t="s">
+        <v>22</v>
+      </c>
+      <c r="N6" s="31"/>
+      <c r="O6" s="32" t="s">
+        <v>23</v>
+      </c>
+      <c r="P6" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q6" s="32" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="18" x14ac:dyDescent="0.3">
+      <c r="A7" s="5"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="H7" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="J7" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="K7" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="L7" s="25"/>
+      <c r="M7" s="26" t="s">
+        <v>16</v>
+      </c>
+      <c r="N7" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="O7" s="33"/>
+      <c r="P7" s="33"/>
+      <c r="Q7" s="33"/>
+    </row>
+    <row r="8" spans="1:17" ht="18" x14ac:dyDescent="0.3">
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+    </row>
+    <row r="9" spans="1:17" ht="18" x14ac:dyDescent="0.35">
+      <c r="A9" s="7"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="13"/>
+      <c r="M9" s="13"/>
+    </row>
+    <row r="10" spans="1:17" ht="18" x14ac:dyDescent="0.35">
+      <c r="A10" s="7"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="13"/>
+      <c r="M10" s="13"/>
+    </row>
+    <row r="11" spans="1:17" ht="18" x14ac:dyDescent="0.35">
+      <c r="A11" s="7"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="13"/>
+      <c r="M11" s="13"/>
+    </row>
+    <row r="12" spans="1:17" ht="18" x14ac:dyDescent="0.35">
+      <c r="A12" s="7"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="13"/>
+      <c r="M12" s="13"/>
+    </row>
+    <row r="13" spans="1:17" ht="18" x14ac:dyDescent="0.35">
+      <c r="A13" s="7"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="13"/>
+      <c r="M13" s="13"/>
+    </row>
+    <row r="14" spans="1:17" ht="18" x14ac:dyDescent="0.35">
+      <c r="A14" s="7"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="13"/>
+      <c r="M14" s="13"/>
+    </row>
+    <row r="15" spans="1:17" ht="18" x14ac:dyDescent="0.35">
+      <c r="A15" s="7"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="13"/>
+      <c r="M15" s="13"/>
+    </row>
+    <row r="16" spans="1:17" ht="18" x14ac:dyDescent="0.35">
+      <c r="A16" s="7"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="13"/>
+      <c r="M16" s="13"/>
     </row>
     <row r="17" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A17" s="11"/>
-      <c r="B17" s="18"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="16"/>
-      <c r="J17" s="15"/>
-      <c r="K17" s="15"/>
-      <c r="L17" s="17"/>
-      <c r="M17" s="17"/>
+      <c r="A17" s="7"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="13"/>
+      <c r="M17" s="13"/>
     </row>
     <row r="18" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A18" s="11"/>
-      <c r="B18" s="18"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="16"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="17"/>
-      <c r="M18" s="17"/>
+      <c r="A18" s="7"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="11"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="13"/>
+      <c r="M18" s="13"/>
     </row>
     <row r="19" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A19" s="11"/>
-      <c r="B19" s="22"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="16"/>
-      <c r="J19" s="15"/>
-      <c r="K19" s="15"/>
-      <c r="L19" s="17"/>
-      <c r="M19" s="17"/>
+      <c r="A19" s="7"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="11"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="13"/>
+      <c r="M19" s="13"/>
     </row>
     <row r="20" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A20" s="11"/>
-      <c r="B20" s="18"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="15"/>
-      <c r="I20" s="16"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="15"/>
-      <c r="L20" s="17"/>
-      <c r="M20" s="17"/>
+      <c r="A20" s="7"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="13"/>
+      <c r="M20" s="13"/>
     </row>
     <row r="21" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A21" s="11"/>
-      <c r="B21" s="18"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
-      <c r="I21" s="16"/>
-      <c r="J21" s="15"/>
-      <c r="K21" s="15"/>
-      <c r="L21" s="17"/>
-      <c r="M21" s="17"/>
+      <c r="A21" s="7"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="11"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="13"/>
+      <c r="M21" s="13"/>
     </row>
     <row r="22" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A22" s="11"/>
-      <c r="B22" s="18"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="16"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="15"/>
-      <c r="L22" s="17"/>
-      <c r="M22" s="17"/>
+      <c r="A22" s="7"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="11"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="13"/>
+      <c r="M22" s="13"/>
     </row>
     <row r="23" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A23" s="11"/>
-      <c r="B23" s="18"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="15"/>
-      <c r="F23" s="15"/>
-      <c r="G23" s="15"/>
-      <c r="H23" s="15"/>
-      <c r="I23" s="16"/>
-      <c r="J23" s="15"/>
-      <c r="K23" s="15"/>
-      <c r="L23" s="17"/>
-      <c r="M23" s="17"/>
+      <c r="A23" s="7"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="11"/>
+      <c r="K23" s="11"/>
+      <c r="L23" s="13"/>
+      <c r="M23" s="13"/>
     </row>
     <row r="24" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A24" s="11"/>
-      <c r="B24" s="18"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="15"/>
-      <c r="I24" s="16"/>
-      <c r="J24" s="15"/>
-      <c r="K24" s="15"/>
-      <c r="L24" s="17"/>
-      <c r="M24" s="17"/>
+      <c r="A24" s="7"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="11"/>
+      <c r="L24" s="13"/>
+      <c r="M24" s="13"/>
     </row>
     <row r="25" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A25" s="11"/>
-      <c r="B25" s="18"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="15"/>
-      <c r="I25" s="16"/>
-      <c r="J25" s="15"/>
-      <c r="K25" s="15"/>
-      <c r="L25" s="17"/>
-      <c r="M25" s="17"/>
+      <c r="A25" s="7"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="11"/>
+      <c r="K25" s="11"/>
+      <c r="L25" s="13"/>
+      <c r="M25" s="13"/>
     </row>
     <row r="26" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A26" s="11"/>
-      <c r="B26" s="18"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="15"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="16"/>
-      <c r="J26" s="15"/>
-      <c r="K26" s="15"/>
-      <c r="L26" s="17"/>
-      <c r="M26" s="17"/>
+      <c r="A26" s="7"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="11"/>
+      <c r="K26" s="11"/>
+      <c r="L26" s="13"/>
+      <c r="M26" s="13"/>
     </row>
     <row r="27" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A27" s="11"/>
-      <c r="B27" s="18"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="15"/>
-      <c r="F27" s="15"/>
-      <c r="G27" s="15"/>
-      <c r="H27" s="15"/>
-      <c r="I27" s="16"/>
-      <c r="J27" s="15"/>
-      <c r="K27" s="15"/>
-      <c r="L27" s="17"/>
-      <c r="M27" s="17"/>
+      <c r="A27" s="7"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="12"/>
+      <c r="J27" s="11"/>
+      <c r="K27" s="11"/>
+      <c r="L27" s="13"/>
+      <c r="M27" s="13"/>
     </row>
     <row r="28" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A28" s="11"/>
-      <c r="B28" s="18"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="15"/>
-      <c r="I28" s="16"/>
-      <c r="J28" s="15"/>
-      <c r="K28" s="15"/>
-      <c r="L28" s="17"/>
-      <c r="M28" s="17"/>
+      <c r="A28" s="7"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="12"/>
+      <c r="J28" s="11"/>
+      <c r="K28" s="11"/>
+      <c r="L28" s="13"/>
+      <c r="M28" s="13"/>
     </row>
     <row r="29" spans="1:13" ht="18" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
@@ -1017,12 +1208,12 @@
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
-      <c r="I30" s="5" t="s">
+      <c r="I30" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="J30" s="5"/>
-      <c r="K30" s="5"/>
-      <c r="L30" s="5"/>
+      <c r="J30" s="19"/>
+      <c r="K30" s="19"/>
+      <c r="L30" s="19"/>
       <c r="M30" s="4"/>
     </row>
     <row r="31" spans="1:13" ht="18" x14ac:dyDescent="0.35">
@@ -1034,12 +1225,12 @@
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
-      <c r="I31" s="6" t="s">
+      <c r="I31" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J31" s="6"/>
-      <c r="K31" s="6"/>
-      <c r="L31" s="6"/>
+      <c r="J31" s="20"/>
+      <c r="K31" s="20"/>
+      <c r="L31" s="20"/>
       <c r="M31" s="4"/>
     </row>
     <row r="32" spans="1:13" ht="18" x14ac:dyDescent="0.35">
@@ -1051,20 +1242,30 @@
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
-      <c r="I32" s="5" t="s">
+      <c r="I32" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="J32" s="5"/>
-      <c r="K32" s="5"/>
-      <c r="L32" s="5"/>
+      <c r="J32" s="19"/>
+      <c r="K32" s="19"/>
+      <c r="L32" s="19"/>
       <c r="M32" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="14">
+    <mergeCell ref="O6:O7"/>
+    <mergeCell ref="P6:P7"/>
+    <mergeCell ref="Q6:Q7"/>
     <mergeCell ref="I30:L30"/>
     <mergeCell ref="I31:L31"/>
     <mergeCell ref="I32:L32"/>
     <mergeCell ref="A1:M1"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="L6:L7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feature: export excel gradetable for a classSubject and for 1 semester of class
</commit_message>
<xml_diff>
--- a/src/assets/bangdiem_template.xlsx
+++ b/src/assets/bangdiem_template.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace\QuanTriTruongHoc_BE\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21EBFD5C-00F7-4AE2-9340-F4844731D463}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7238538C-2122-45F4-9FCF-CEADE311AD7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5E6F906E-4952-4227-9D02-B0001F3530D5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{5E6F906E-4952-4227-9D02-B0001F3530D5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Tổng kết" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
   <si>
     <t xml:space="preserve">KẾT QUẢ HỌC TẬP MÔN HỌC/MÔ ĐUN
 TIN HỌC VĂN PHÒNG        </t>
@@ -64,9 +65,6 @@
     <t>Khóa: {{batchCode}}</t>
   </si>
   <si>
-    <t>Lớp: {{courseOfferName}}</t>
-  </si>
-  <si>
     <t>MSSV</t>
   </si>
   <si>
@@ -104,6 +102,49 @@
   </si>
   <si>
     <t>Ghi chú</t>
+  </si>
+  <si>
+    <t>Lớp: {{className}}</t>
+  </si>
+  <si>
+    <t>{{subjectName}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KẾT QUẢ HỌC TẬP MÔN HỌC/MÔ ĐUN
+HỌC KỲ 1 NĂM HỌC: 2024 - 2025       </t>
+  </si>
+  <si>
+    <t>Tên môn học</t>
+  </si>
+  <si>
+    <t>Họ và tên học sinh</t>
+  </si>
+  <si>
+    <t>Điểm TB
+(hệ 10)</t>
+  </si>
+  <si>
+    <t>Điểm TB
+(hệ 4)</t>
+  </si>
+  <si>
+    <t>Điểm chữ</t>
+  </si>
+  <si>
+    <t>Xếp loại HL</t>
+  </si>
+  <si>
+    <t>Xếp loại RL</t>
+  </si>
+  <si>
+    <t>Xếp loại RL
+(điểm)</t>
+  </si>
+  <si>
+    <t>{{semesterName}}</t>
+  </si>
+  <si>
+    <t>MSV</t>
   </si>
 </sst>
 </file>
@@ -113,7 +154,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,6 +205,43 @@
       <family val="1"/>
       <scheme val="major"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri Light"/>
+      <family val="1"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri Light"/>
+      <family val="1"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri Light"/>
+      <family val="1"/>
+      <scheme val="major"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -173,7 +251,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -269,11 +347,51 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -327,54 +445,129 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{5F32061F-8A45-49D2-869F-85F4F33E0B02}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -686,7 +879,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{126F2789-0FE7-4317-A3A6-DB05700D32CA}">
-  <dimension ref="A1:Q32"/>
+  <dimension ref="A1:Q33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="21.44140625" customWidth="1"/>
@@ -696,68 +889,67 @@
     <col min="8" max="8" width="8.109375" customWidth="1"/>
     <col min="10" max="10" width="8.77734375" customWidth="1"/>
     <col min="12" max="12" width="12.33203125" customWidth="1"/>
-    <col min="15" max="15" width="15.109375" customWidth="1"/>
-    <col min="16" max="16" width="13.6640625" customWidth="1"/>
+    <col min="15" max="15" width="17.33203125" customWidth="1"/>
+    <col min="16" max="16" width="16.6640625" customWidth="1"/>
+    <col min="17" max="17" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-    </row>
-    <row r="2" spans="1:17" ht="18" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="1" t="s">
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
+      <c r="G1" s="49"/>
+      <c r="H1" s="49"/>
+      <c r="I1" s="49"/>
+      <c r="J1" s="49"/>
+      <c r="K1" s="49"/>
+      <c r="L1" s="49"/>
+      <c r="M1" s="49"/>
+    </row>
+    <row r="2" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="A2" s="48" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="48"/>
+      <c r="L2" s="48"/>
+      <c r="M2" s="19"/>
+    </row>
+    <row r="3" spans="1:17" ht="18" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-    </row>
-    <row r="3" spans="1:17" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+    </row>
+    <row r="4" spans="1:17" ht="18" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-    </row>
-    <row r="4" spans="1:17" ht="18" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -768,14 +960,16 @@
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
     </row>
     <row r="5" spans="1:17" ht="18" x14ac:dyDescent="0.35">
-      <c r="A5" s="1"/>
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -784,122 +978,124 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
+      <c r="J5" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
     </row>
-    <row r="6" spans="1:17" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+    <row r="6" spans="1:17" ht="18" x14ac:dyDescent="0.35">
+      <c r="A6" s="1"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+    </row>
+    <row r="7" spans="1:17" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B7" s="50" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="23" t="s">
+      <c r="D7" s="50" t="s">
+        <v>2</v>
+      </c>
+      <c r="E7" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="23" t="s">
-        <v>2</v>
-      </c>
-      <c r="E6" s="23" t="s">
+      <c r="F7" s="50"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="51" t="s">
+        <v>18</v>
+      </c>
+      <c r="I7" s="52"/>
+      <c r="J7" s="52"/>
+      <c r="K7" s="53"/>
+      <c r="L7" s="51" t="s">
+        <v>20</v>
+      </c>
+      <c r="M7" s="51" t="s">
+        <v>21</v>
+      </c>
+      <c r="N7" s="53"/>
+      <c r="O7" s="56" t="s">
+        <v>22</v>
+      </c>
+      <c r="P7" s="56" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q7" s="56" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" ht="18" x14ac:dyDescent="0.3">
+      <c r="A8" s="54"/>
+      <c r="B8" s="54"/>
+      <c r="C8" s="54"/>
+      <c r="D8" s="55"/>
+      <c r="E8" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="23"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="29" t="s">
+      <c r="F8" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="K8" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="30"/>
-      <c r="J6" s="30"/>
-      <c r="K6" s="31"/>
-      <c r="L6" s="29" t="s">
-        <v>21</v>
-      </c>
-      <c r="M6" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="N6" s="31"/>
-      <c r="O6" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="P6" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q6" s="32" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" ht="18" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="26" t="s">
+      <c r="L8" s="55"/>
+      <c r="M8" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="N8" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="27" t="s">
-        <v>17</v>
-      </c>
-      <c r="G7" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="H7" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="I7" s="27" t="s">
-        <v>17</v>
-      </c>
-      <c r="J7" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="K7" s="28" t="s">
-        <v>20</v>
-      </c>
-      <c r="L7" s="25"/>
-      <c r="M7" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="N7" s="28" t="s">
-        <v>17</v>
-      </c>
-      <c r="O7" s="33"/>
-      <c r="P7" s="33"/>
-      <c r="Q7" s="33"/>
-    </row>
-    <row r="8" spans="1:17" ht="18" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
-    </row>
-    <row r="9" spans="1:17" ht="18" x14ac:dyDescent="0.35">
-      <c r="A9" s="7"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="13"/>
-      <c r="M9" s="13"/>
+      <c r="O8" s="57"/>
+      <c r="P8" s="57"/>
+      <c r="Q8" s="57"/>
+    </row>
+    <row r="9" spans="1:17" ht="18" x14ac:dyDescent="0.3">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
     </row>
     <row r="10" spans="1:17" ht="18" x14ac:dyDescent="0.35">
       <c r="A10" s="7"/>
-      <c r="B10" s="14"/>
+      <c r="B10" s="8"/>
       <c r="C10" s="9"/>
       <c r="D10" s="10"/>
       <c r="E10" s="11"/>
@@ -929,7 +1125,7 @@
     </row>
     <row r="12" spans="1:17" ht="18" x14ac:dyDescent="0.35">
       <c r="A12" s="7"/>
-      <c r="B12" s="8"/>
+      <c r="B12" s="14"/>
       <c r="C12" s="9"/>
       <c r="D12" s="10"/>
       <c r="E12" s="11"/>
@@ -944,8 +1140,8 @@
     </row>
     <row r="13" spans="1:17" ht="18" x14ac:dyDescent="0.35">
       <c r="A13" s="7"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="16"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="9"/>
       <c r="D13" s="10"/>
       <c r="E13" s="11"/>
       <c r="F13" s="11"/>
@@ -989,7 +1185,7 @@
     </row>
     <row r="16" spans="1:17" ht="18" x14ac:dyDescent="0.35">
       <c r="A16" s="7"/>
-      <c r="B16" s="17"/>
+      <c r="B16" s="15"/>
       <c r="C16" s="16"/>
       <c r="D16" s="10"/>
       <c r="E16" s="11"/>
@@ -1004,8 +1200,8 @@
     </row>
     <row r="17" spans="1:13" ht="18" x14ac:dyDescent="0.35">
       <c r="A17" s="7"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="9"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="16"/>
       <c r="D17" s="10"/>
       <c r="E17" s="11"/>
       <c r="F17" s="11"/>
@@ -1034,7 +1230,7 @@
     </row>
     <row r="19" spans="1:13" ht="18" x14ac:dyDescent="0.35">
       <c r="A19" s="7"/>
-      <c r="B19" s="18"/>
+      <c r="B19" s="14"/>
       <c r="C19" s="9"/>
       <c r="D19" s="10"/>
       <c r="E19" s="11"/>
@@ -1049,7 +1245,7 @@
     </row>
     <row r="20" spans="1:13" ht="18" x14ac:dyDescent="0.35">
       <c r="A20" s="7"/>
-      <c r="B20" s="14"/>
+      <c r="B20" s="18"/>
       <c r="C20" s="9"/>
       <c r="D20" s="10"/>
       <c r="E20" s="11"/>
@@ -1183,24 +1379,24 @@
       <c r="M28" s="13"/>
     </row>
     <row r="29" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="7"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="11"/>
+      <c r="G29" s="11"/>
+      <c r="H29" s="11"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="11"/>
+      <c r="K29" s="11"/>
+      <c r="L29" s="13"/>
+      <c r="M29" s="13"/>
+    </row>
+    <row r="30" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+      <c r="A30" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4"/>
-      <c r="L29" s="4"/>
-      <c r="M29" s="4"/>
-    </row>
-    <row r="30" spans="1:13" ht="18" x14ac:dyDescent="0.35">
-      <c r="A30" s="4"/>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -1208,12 +1404,10 @@
       <c r="F30" s="4"/>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
-      <c r="I30" s="19" t="s">
-        <v>4</v>
-      </c>
-      <c r="J30" s="19"/>
-      <c r="K30" s="19"/>
-      <c r="L30" s="19"/>
+      <c r="I30" s="4"/>
+      <c r="J30" s="4"/>
+      <c r="K30" s="4"/>
+      <c r="L30" s="4"/>
       <c r="M30" s="4"/>
     </row>
     <row r="31" spans="1:13" ht="18" x14ac:dyDescent="0.35">
@@ -1225,12 +1419,12 @@
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
-      <c r="I31" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="J31" s="20"/>
-      <c r="K31" s="20"/>
-      <c r="L31" s="20"/>
+      <c r="I31" s="47" t="s">
+        <v>4</v>
+      </c>
+      <c r="J31" s="47"/>
+      <c r="K31" s="47"/>
+      <c r="L31" s="47"/>
       <c r="M31" s="4"/>
     </row>
     <row r="32" spans="1:13" ht="18" x14ac:dyDescent="0.35">
@@ -1242,30 +1436,474 @@
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
-      <c r="I32" s="19" t="s">
+      <c r="I32" s="58" t="s">
+        <v>5</v>
+      </c>
+      <c r="J32" s="58"/>
+      <c r="K32" s="58"/>
+      <c r="L32" s="58"/>
+      <c r="M32" s="4"/>
+    </row>
+    <row r="33" spans="1:13" ht="18" x14ac:dyDescent="0.35">
+      <c r="A33" s="4"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="J32" s="19"/>
-      <c r="K32" s="19"/>
-      <c r="L32" s="19"/>
-      <c r="M32" s="4"/>
+      <c r="J33" s="47"/>
+      <c r="K33" s="47"/>
+      <c r="L33" s="47"/>
+      <c r="M33" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="P7:P8"/>
+    <mergeCell ref="Q7:Q8"/>
+    <mergeCell ref="I31:L31"/>
+    <mergeCell ref="I32:L32"/>
+    <mergeCell ref="I33:L33"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="E7:G7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A7:A8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAC81119-177E-4927-B07A-47D1C63713F2}">
+  <dimension ref="A1:O26"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="21.88671875" customWidth="1"/>
+    <col min="4" max="4" width="19.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="A1" s="38" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="38"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+    </row>
+    <row r="2" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="A2" s="43" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+    </row>
+    <row r="3" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="29"/>
+      <c r="B3" s="29"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="42" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="42"/>
+      <c r="K3" s="31" t="s">
+        <v>26</v>
+      </c>
+      <c r="L3" s="32"/>
+    </row>
+    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="40" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="44" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="44" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="41" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="41" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" s="41" t="s">
+        <v>32</v>
+      </c>
+      <c r="H4" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" s="41" t="s">
+        <v>34</v>
+      </c>
+      <c r="J4" s="41" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4" s="33"/>
+      <c r="L4" s="41" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="40"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="41"/>
+      <c r="I5" s="41"/>
+      <c r="J5" s="41"/>
+      <c r="K5" s="33"/>
+      <c r="L5" s="41"/>
+    </row>
+    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="40"/>
+      <c r="B6" s="46"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="40"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="41"/>
+      <c r="K6" s="33"/>
+      <c r="L6" s="41"/>
+    </row>
+    <row r="7" spans="1:15" ht="18" x14ac:dyDescent="0.3">
+      <c r="A7" s="24"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="34"/>
+      <c r="K7" s="34"/>
+      <c r="L7" s="34"/>
+    </row>
+    <row r="8" spans="1:15" ht="18" x14ac:dyDescent="0.3">
+      <c r="A8" s="24"/>
+      <c r="B8" s="37"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="34"/>
+      <c r="J8" s="34"/>
+      <c r="K8" s="34"/>
+      <c r="L8" s="34"/>
+      <c r="O8" s="59"/>
+    </row>
+    <row r="9" spans="1:15" ht="18" x14ac:dyDescent="0.3">
+      <c r="A9" s="24"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="34"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="34"/>
+      <c r="I9" s="34"/>
+      <c r="J9" s="34"/>
+      <c r="K9" s="34"/>
+      <c r="L9" s="34"/>
+    </row>
+    <row r="10" spans="1:15" ht="18" x14ac:dyDescent="0.3">
+      <c r="A10" s="24"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="34"/>
+      <c r="I10" s="34"/>
+      <c r="J10" s="34"/>
+      <c r="K10" s="34"/>
+      <c r="L10" s="34"/>
+    </row>
+    <row r="11" spans="1:15" ht="18" x14ac:dyDescent="0.3">
+      <c r="A11" s="24"/>
+      <c r="B11" s="37"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="34"/>
+      <c r="I11" s="34"/>
+      <c r="J11" s="34"/>
+      <c r="K11" s="34"/>
+      <c r="L11" s="34"/>
+    </row>
+    <row r="12" spans="1:15" ht="18" x14ac:dyDescent="0.3">
+      <c r="A12" s="24"/>
+      <c r="B12" s="37"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
+      <c r="H12" s="34"/>
+      <c r="I12" s="34"/>
+      <c r="J12" s="34"/>
+      <c r="K12" s="34"/>
+      <c r="L12" s="34"/>
+    </row>
+    <row r="13" spans="1:15" ht="18" x14ac:dyDescent="0.3">
+      <c r="A13" s="24"/>
+      <c r="B13" s="37"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="34"/>
+      <c r="J13" s="34"/>
+      <c r="K13" s="34"/>
+      <c r="L13" s="34"/>
+    </row>
+    <row r="14" spans="1:15" ht="18" x14ac:dyDescent="0.3">
+      <c r="A14" s="24"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="34"/>
+      <c r="I14" s="34"/>
+      <c r="J14" s="34"/>
+      <c r="K14" s="34"/>
+      <c r="L14" s="34"/>
+    </row>
+    <row r="15" spans="1:15" ht="18" x14ac:dyDescent="0.3">
+      <c r="A15" s="24"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="34"/>
+      <c r="I15" s="34"/>
+      <c r="J15" s="34"/>
+      <c r="K15" s="34"/>
+      <c r="L15" s="34"/>
+    </row>
+    <row r="16" spans="1:15" ht="18" x14ac:dyDescent="0.3">
+      <c r="A16" s="24"/>
+      <c r="B16" s="37"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="34"/>
+      <c r="I16" s="34"/>
+      <c r="J16" s="34"/>
+      <c r="K16" s="34"/>
+      <c r="L16" s="34"/>
+    </row>
+    <row r="17" spans="1:12" ht="18" x14ac:dyDescent="0.3">
+      <c r="A17" s="24"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="34"/>
+      <c r="I17" s="34"/>
+      <c r="J17" s="34"/>
+      <c r="K17" s="34"/>
+      <c r="L17" s="34"/>
+    </row>
+    <row r="18" spans="1:12" ht="18" x14ac:dyDescent="0.3">
+      <c r="A18" s="24"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+      <c r="I18" s="34"/>
+      <c r="J18" s="34"/>
+      <c r="K18" s="34"/>
+      <c r="L18" s="34"/>
+    </row>
+    <row r="19" spans="1:12" ht="18" x14ac:dyDescent="0.3">
+      <c r="A19" s="24"/>
+      <c r="B19" s="37"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+      <c r="I19" s="34"/>
+      <c r="J19" s="34"/>
+      <c r="K19" s="34"/>
+      <c r="L19" s="34"/>
+    </row>
+    <row r="20" spans="1:12" ht="18" x14ac:dyDescent="0.3">
+      <c r="A20" s="24"/>
+      <c r="B20" s="37"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="34"/>
+      <c r="I20" s="34"/>
+      <c r="J20" s="34"/>
+      <c r="K20" s="34"/>
+      <c r="L20" s="34"/>
+    </row>
+    <row r="21" spans="1:12" ht="18" x14ac:dyDescent="0.3">
+      <c r="A21" s="24"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="34"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="34"/>
+      <c r="I21" s="34"/>
+      <c r="J21" s="34"/>
+      <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
+    </row>
+    <row r="22" spans="1:12" ht="18" x14ac:dyDescent="0.3">
+      <c r="A22" s="24"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="34"/>
+      <c r="I22" s="34"/>
+      <c r="J22" s="34"/>
+      <c r="K22" s="34"/>
+      <c r="L22" s="34"/>
+    </row>
+    <row r="23" spans="1:12" ht="18" x14ac:dyDescent="0.3">
+      <c r="A23" s="24"/>
+      <c r="B23" s="37"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="34"/>
+      <c r="F23" s="34"/>
+      <c r="G23" s="34"/>
+      <c r="H23" s="34"/>
+      <c r="I23" s="34"/>
+      <c r="J23" s="34"/>
+      <c r="K23" s="34"/>
+      <c r="L23" s="34"/>
+    </row>
+    <row r="24" spans="1:12" ht="18" x14ac:dyDescent="0.3">
+      <c r="A24" s="24"/>
+      <c r="B24" s="37"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="34"/>
+      <c r="F24" s="34"/>
+      <c r="G24" s="34"/>
+      <c r="H24" s="34"/>
+      <c r="I24" s="34"/>
+      <c r="J24" s="34"/>
+      <c r="K24" s="34"/>
+      <c r="L24" s="34"/>
+    </row>
+    <row r="25" spans="1:12" ht="18" x14ac:dyDescent="0.3">
+      <c r="A25" s="24"/>
+      <c r="B25" s="37"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="34"/>
+      <c r="F25" s="34"/>
+      <c r="G25" s="34"/>
+      <c r="H25" s="34"/>
+      <c r="I25" s="34"/>
+      <c r="J25" s="34"/>
+      <c r="K25" s="34"/>
+      <c r="L25" s="34"/>
+    </row>
+    <row r="26" spans="1:12" ht="18" x14ac:dyDescent="0.3">
+      <c r="A26" s="24"/>
+      <c r="B26" s="37"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="34"/>
+      <c r="I26" s="34"/>
+      <c r="J26" s="34"/>
+      <c r="K26" s="34"/>
+      <c r="L26" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="O6:O7"/>
-    <mergeCell ref="P6:P7"/>
-    <mergeCell ref="Q6:Q7"/>
-    <mergeCell ref="I30:L30"/>
-    <mergeCell ref="I31:L31"/>
-    <mergeCell ref="I32:L32"/>
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="L6:L7"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="D4:D6"/>
+    <mergeCell ref="H4:H6"/>
+    <mergeCell ref="I3:J3"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="L4:L6"/>
+    <mergeCell ref="E4:E6"/>
+    <mergeCell ref="F4:F6"/>
+    <mergeCell ref="G4:G6"/>
+    <mergeCell ref="I4:I6"/>
+    <mergeCell ref="J4:J6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update: update export file tongket
</commit_message>
<xml_diff>
--- a/src/assets/bangdiem_template.xlsx
+++ b/src/assets/bangdiem_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WorkSpace\QuanTriTruongHoc_BE\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7238538C-2122-45F4-9FCF-CEADE311AD7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C16F822-3589-4AFB-9994-86F241E592AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{5E6F906E-4952-4227-9D02-B0001F3530D5}"/>
   </bookViews>
@@ -251,7 +251,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -354,19 +354,6 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -391,7 +378,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -460,46 +447,48 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -509,27 +498,42 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -554,16 +558,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -895,37 +889,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="55" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
-      <c r="L1" s="49"/>
-      <c r="M1" s="49"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
+      <c r="G1" s="56"/>
+      <c r="H1" s="56"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
+      <c r="L1" s="56"/>
+      <c r="M1" s="56"/>
     </row>
     <row r="2" spans="1:17" ht="21" x14ac:dyDescent="0.3">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
-      <c r="L2" s="48"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
+      <c r="K2" s="55"/>
+      <c r="L2" s="55"/>
       <c r="M2" s="19"/>
     </row>
     <row r="3" spans="1:17" ht="18" x14ac:dyDescent="0.3">
@@ -1001,51 +995,51 @@
       <c r="M6" s="3"/>
     </row>
     <row r="7" spans="1:17" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="50" t="s">
+      <c r="A7" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="50" t="s">
+      <c r="B7" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="50" t="s">
+      <c r="C7" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="50" t="s">
+      <c r="D7" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="50" t="s">
+      <c r="E7" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="50"/>
-      <c r="G7" s="51"/>
-      <c r="H7" s="51" t="s">
+      <c r="F7" s="57"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="58" t="s">
         <v>18</v>
       </c>
-      <c r="I7" s="52"/>
-      <c r="J7" s="52"/>
-      <c r="K7" s="53"/>
-      <c r="L7" s="51" t="s">
+      <c r="I7" s="59"/>
+      <c r="J7" s="59"/>
+      <c r="K7" s="60"/>
+      <c r="L7" s="58" t="s">
         <v>20</v>
       </c>
-      <c r="M7" s="51" t="s">
+      <c r="M7" s="58" t="s">
         <v>21</v>
       </c>
-      <c r="N7" s="53"/>
-      <c r="O7" s="56" t="s">
+      <c r="N7" s="60"/>
+      <c r="O7" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="P7" s="56" t="s">
+      <c r="P7" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="Q7" s="56" t="s">
+      <c r="Q7" s="51" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="18" x14ac:dyDescent="0.3">
-      <c r="A8" s="54"/>
-      <c r="B8" s="54"/>
-      <c r="C8" s="54"/>
-      <c r="D8" s="55"/>
+      <c r="A8" s="61"/>
+      <c r="B8" s="61"/>
+      <c r="C8" s="61"/>
+      <c r="D8" s="62"/>
       <c r="E8" s="20" t="s">
         <v>15</v>
       </c>
@@ -1067,16 +1061,16 @@
       <c r="K8" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="L8" s="55"/>
+      <c r="L8" s="62"/>
       <c r="M8" s="20" t="s">
         <v>15</v>
       </c>
       <c r="N8" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="57"/>
-      <c r="P8" s="57"/>
-      <c r="Q8" s="57"/>
+      <c r="O8" s="52"/>
+      <c r="P8" s="52"/>
+      <c r="Q8" s="52"/>
     </row>
     <row r="9" spans="1:17" ht="18" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
@@ -1419,12 +1413,12 @@
       <c r="F31" s="4"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
-      <c r="I31" s="47" t="s">
+      <c r="I31" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="J31" s="47"/>
-      <c r="K31" s="47"/>
-      <c r="L31" s="47"/>
+      <c r="J31" s="53"/>
+      <c r="K31" s="53"/>
+      <c r="L31" s="53"/>
       <c r="M31" s="4"/>
     </row>
     <row r="32" spans="1:13" ht="18" x14ac:dyDescent="0.35">
@@ -1436,12 +1430,12 @@
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
-      <c r="I32" s="58" t="s">
+      <c r="I32" s="54" t="s">
         <v>5</v>
       </c>
-      <c r="J32" s="58"/>
-      <c r="K32" s="58"/>
-      <c r="L32" s="58"/>
+      <c r="J32" s="54"/>
+      <c r="K32" s="54"/>
+      <c r="L32" s="54"/>
       <c r="M32" s="4"/>
     </row>
     <row r="33" spans="1:13" ht="18" x14ac:dyDescent="0.35">
@@ -1453,21 +1447,16 @@
       <c r="F33" s="4"/>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
-      <c r="I33" s="47" t="s">
+      <c r="I33" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="J33" s="47"/>
-      <c r="K33" s="47"/>
-      <c r="L33" s="47"/>
+      <c r="J33" s="53"/>
+      <c r="K33" s="53"/>
+      <c r="L33" s="53"/>
       <c r="M33" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="O7:O8"/>
-    <mergeCell ref="P7:P8"/>
-    <mergeCell ref="Q7:Q8"/>
-    <mergeCell ref="I31:L31"/>
-    <mergeCell ref="I32:L32"/>
     <mergeCell ref="I33:L33"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="E7:G7"/>
@@ -1479,6 +1468,11 @@
     <mergeCell ref="L7:L8"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A7:A8"/>
+    <mergeCell ref="O7:O8"/>
+    <mergeCell ref="P7:P8"/>
+    <mergeCell ref="Q7:Q8"/>
+    <mergeCell ref="I31:L31"/>
+    <mergeCell ref="I32:L32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1489,407 +1483,408 @@
   <dimension ref="A1:O26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="21.88671875" customWidth="1"/>
-    <col min="4" max="4" width="19.77734375" customWidth="1"/>
+    <col min="2" max="2" width="17.88671875" customWidth="1"/>
+    <col min="3" max="3" width="31.5546875" customWidth="1"/>
+    <col min="4" max="4" width="22.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
       <c r="K1" s="23"/>
       <c r="L1" s="23"/>
     </row>
     <row r="2" spans="1:15" ht="21" x14ac:dyDescent="0.3">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="47" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="43"/>
-      <c r="L2" s="43"/>
-    </row>
-    <row r="3" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="29"/>
-      <c r="B3" s="29"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="42" t="s">
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+    </row>
+    <row r="3" spans="1:15" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="24"/>
+      <c r="B3" s="24"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="J3" s="42"/>
-      <c r="K3" s="31" t="s">
+      <c r="J3" s="46"/>
+      <c r="K3" s="49" t="s">
         <v>26</v>
       </c>
-      <c r="L3" s="32"/>
+      <c r="L3" s="26"/>
     </row>
     <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="40" t="s">
+      <c r="A4" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="44" t="s">
+      <c r="B4" s="43" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="44" t="s">
+      <c r="C4" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="40" t="s">
+      <c r="D4" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="41" t="s">
+      <c r="E4" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="F4" s="41" t="s">
+      <c r="F4" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="G4" s="41" t="s">
+      <c r="G4" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="H4" s="41" t="s">
+      <c r="H4" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="I4" s="41" t="s">
+      <c r="I4" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="J4" s="41" t="s">
+      <c r="J4" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="K4" s="33"/>
-      <c r="L4" s="41" t="s">
+      <c r="K4" s="50"/>
+      <c r="L4" s="44" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="40"/>
-      <c r="B5" s="45"/>
-      <c r="C5" s="45"/>
-      <c r="D5" s="40"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="41"/>
-      <c r="I5" s="41"/>
-      <c r="J5" s="41"/>
-      <c r="K5" s="33"/>
-      <c r="L5" s="41"/>
+      <c r="A5" s="42"/>
+      <c r="B5" s="48"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+      <c r="K5" s="50"/>
+      <c r="L5" s="44"/>
     </row>
     <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="40"/>
-      <c r="B6" s="46"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="41"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="41"/>
-      <c r="I6" s="41"/>
-      <c r="J6" s="41"/>
-      <c r="K6" s="33"/>
-      <c r="L6" s="41"/>
+      <c r="A6" s="43"/>
+      <c r="B6" s="48"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="45"/>
+      <c r="G6" s="45"/>
+      <c r="H6" s="45"/>
+      <c r="I6" s="45"/>
+      <c r="J6" s="45"/>
+      <c r="K6" s="50"/>
+      <c r="L6" s="45"/>
     </row>
     <row r="7" spans="1:15" ht="18" x14ac:dyDescent="0.3">
-      <c r="A7" s="24"/>
-      <c r="B7" s="37"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="34"/>
-      <c r="F7" s="34"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="34"/>
-      <c r="I7" s="34"/>
-      <c r="J7" s="34"/>
-      <c r="K7" s="34"/>
-      <c r="L7" s="34"/>
+      <c r="A7" s="36"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="39"/>
+      <c r="H7" s="39"/>
+      <c r="I7" s="39"/>
+      <c r="J7" s="39"/>
+      <c r="K7" s="39"/>
+      <c r="L7" s="39"/>
     </row>
     <row r="8" spans="1:15" ht="18" x14ac:dyDescent="0.3">
-      <c r="A8" s="24"/>
-      <c r="B8" s="37"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="34"/>
-      <c r="J8" s="34"/>
-      <c r="K8" s="34"/>
-      <c r="L8" s="34"/>
-      <c r="O8" s="59"/>
+      <c r="A8" s="28"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="31"/>
+      <c r="F8" s="31"/>
+      <c r="G8" s="31"/>
+      <c r="H8" s="31"/>
+      <c r="I8" s="31"/>
+      <c r="J8" s="31"/>
+      <c r="K8" s="31"/>
+      <c r="L8" s="31"/>
+      <c r="O8" s="27"/>
     </row>
     <row r="9" spans="1:15" ht="18" x14ac:dyDescent="0.3">
-      <c r="A9" s="24"/>
-      <c r="B9" s="37"/>
-      <c r="C9" s="27"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
-      <c r="G9" s="34"/>
-      <c r="H9" s="34"/>
-      <c r="I9" s="34"/>
-      <c r="J9" s="34"/>
-      <c r="K9" s="34"/>
-      <c r="L9" s="34"/>
+      <c r="A9" s="28"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="32"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="31"/>
+      <c r="F9" s="31"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
+      <c r="J9" s="31"/>
+      <c r="K9" s="31"/>
+      <c r="L9" s="31"/>
     </row>
     <row r="10" spans="1:15" ht="18" x14ac:dyDescent="0.3">
-      <c r="A10" s="24"/>
-      <c r="B10" s="37"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="26"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="34"/>
-      <c r="I10" s="34"/>
-      <c r="J10" s="34"/>
-      <c r="K10" s="34"/>
-      <c r="L10" s="34"/>
+      <c r="A10" s="28"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="31"/>
+      <c r="L10" s="31"/>
     </row>
     <row r="11" spans="1:15" ht="18" x14ac:dyDescent="0.3">
-      <c r="A11" s="24"/>
-      <c r="B11" s="37"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="34"/>
-      <c r="H11" s="34"/>
-      <c r="I11" s="34"/>
-      <c r="J11" s="34"/>
-      <c r="K11" s="34"/>
-      <c r="L11" s="34"/>
+      <c r="A11" s="28"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="30"/>
+      <c r="E11" s="31"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="31"/>
+      <c r="J11" s="31"/>
+      <c r="K11" s="31"/>
+      <c r="L11" s="31"/>
     </row>
     <row r="12" spans="1:15" ht="18" x14ac:dyDescent="0.3">
-      <c r="A12" s="24"/>
-      <c r="B12" s="37"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="34"/>
-      <c r="G12" s="34"/>
-      <c r="H12" s="34"/>
-      <c r="I12" s="34"/>
-      <c r="J12" s="34"/>
-      <c r="K12" s="34"/>
-      <c r="L12" s="34"/>
+      <c r="A12" s="28"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="31"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="31"/>
+      <c r="I12" s="31"/>
+      <c r="J12" s="31"/>
+      <c r="K12" s="31"/>
+      <c r="L12" s="31"/>
     </row>
     <row r="13" spans="1:15" ht="18" x14ac:dyDescent="0.3">
-      <c r="A13" s="24"/>
-      <c r="B13" s="37"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="34"/>
-      <c r="I13" s="34"/>
-      <c r="J13" s="34"/>
-      <c r="K13" s="34"/>
-      <c r="L13" s="34"/>
+      <c r="A13" s="28"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
+      <c r="I13" s="31"/>
+      <c r="J13" s="31"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="31"/>
     </row>
     <row r="14" spans="1:15" ht="18" x14ac:dyDescent="0.3">
-      <c r="A14" s="24"/>
-      <c r="B14" s="37"/>
-      <c r="C14" s="36"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="34"/>
-      <c r="I14" s="34"/>
-      <c r="J14" s="34"/>
-      <c r="K14" s="34"/>
-      <c r="L14" s="34"/>
+      <c r="A14" s="28"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="31"/>
+      <c r="I14" s="31"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="31"/>
     </row>
     <row r="15" spans="1:15" ht="18" x14ac:dyDescent="0.3">
-      <c r="A15" s="24"/>
-      <c r="B15" s="37"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="34"/>
-      <c r="I15" s="34"/>
-      <c r="J15" s="34"/>
-      <c r="K15" s="34"/>
-      <c r="L15" s="34"/>
+      <c r="A15" s="28"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="31"/>
+      <c r="H15" s="31"/>
+      <c r="I15" s="31"/>
+      <c r="J15" s="31"/>
+      <c r="K15" s="31"/>
+      <c r="L15" s="31"/>
     </row>
     <row r="16" spans="1:15" ht="18" x14ac:dyDescent="0.3">
-      <c r="A16" s="24"/>
-      <c r="B16" s="37"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="34"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="34"/>
-      <c r="I16" s="34"/>
-      <c r="J16" s="34"/>
-      <c r="K16" s="34"/>
-      <c r="L16" s="34"/>
+      <c r="A16" s="28"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="31"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="31"/>
+      <c r="L16" s="31"/>
     </row>
     <row r="17" spans="1:12" ht="18" x14ac:dyDescent="0.3">
-      <c r="A17" s="24"/>
-      <c r="B17" s="37"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="34"/>
-      <c r="I17" s="34"/>
-      <c r="J17" s="34"/>
-      <c r="K17" s="34"/>
-      <c r="L17" s="34"/>
+      <c r="A17" s="28"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="35"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="31"/>
+      <c r="G17" s="31"/>
+      <c r="H17" s="31"/>
+      <c r="I17" s="31"/>
+      <c r="J17" s="31"/>
+      <c r="K17" s="31"/>
+      <c r="L17" s="31"/>
     </row>
     <row r="18" spans="1:12" ht="18" x14ac:dyDescent="0.3">
-      <c r="A18" s="24"/>
-      <c r="B18" s="37"/>
-      <c r="C18" s="27"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="34"/>
-      <c r="G18" s="34"/>
-      <c r="H18" s="34"/>
-      <c r="I18" s="34"/>
-      <c r="J18" s="34"/>
-      <c r="K18" s="34"/>
-      <c r="L18" s="34"/>
+      <c r="A18" s="28"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="31"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="31"/>
+      <c r="L18" s="31"/>
     </row>
     <row r="19" spans="1:12" ht="18" x14ac:dyDescent="0.3">
-      <c r="A19" s="24"/>
-      <c r="B19" s="37"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="34"/>
-      <c r="I19" s="34"/>
-      <c r="J19" s="34"/>
-      <c r="K19" s="34"/>
-      <c r="L19" s="34"/>
+      <c r="A19" s="28"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="32"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="31"/>
+      <c r="G19" s="31"/>
+      <c r="H19" s="31"/>
+      <c r="I19" s="31"/>
+      <c r="J19" s="31"/>
+      <c r="K19" s="31"/>
+      <c r="L19" s="31"/>
     </row>
     <row r="20" spans="1:12" ht="18" x14ac:dyDescent="0.3">
-      <c r="A20" s="24"/>
-      <c r="B20" s="37"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="34"/>
-      <c r="F20" s="34"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="34"/>
-      <c r="I20" s="34"/>
-      <c r="J20" s="34"/>
-      <c r="K20" s="34"/>
-      <c r="L20" s="34"/>
+      <c r="A20" s="28"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="32"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="31"/>
+      <c r="G20" s="31"/>
+      <c r="H20" s="31"/>
+      <c r="I20" s="31"/>
+      <c r="J20" s="31"/>
+      <c r="K20" s="31"/>
+      <c r="L20" s="31"/>
     </row>
     <row r="21" spans="1:12" ht="18" x14ac:dyDescent="0.3">
-      <c r="A21" s="24"/>
-      <c r="B21" s="37"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="34"/>
-      <c r="J21" s="34"/>
-      <c r="K21" s="34"/>
-      <c r="L21" s="34"/>
+      <c r="A21" s="28"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="31"/>
+      <c r="J21" s="31"/>
+      <c r="K21" s="31"/>
+      <c r="L21" s="31"/>
     </row>
     <row r="22" spans="1:12" ht="18" x14ac:dyDescent="0.3">
-      <c r="A22" s="24"/>
-      <c r="B22" s="37"/>
-      <c r="C22" s="27"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="34"/>
-      <c r="I22" s="34"/>
-      <c r="J22" s="34"/>
-      <c r="K22" s="34"/>
-      <c r="L22" s="34"/>
+      <c r="A22" s="28"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="31"/>
+      <c r="G22" s="31"/>
+      <c r="H22" s="31"/>
+      <c r="I22" s="31"/>
+      <c r="J22" s="31"/>
+      <c r="K22" s="31"/>
+      <c r="L22" s="31"/>
     </row>
     <row r="23" spans="1:12" ht="18" x14ac:dyDescent="0.3">
-      <c r="A23" s="24"/>
-      <c r="B23" s="37"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="34"/>
-      <c r="F23" s="34"/>
-      <c r="G23" s="34"/>
-      <c r="H23" s="34"/>
-      <c r="I23" s="34"/>
-      <c r="J23" s="34"/>
-      <c r="K23" s="34"/>
-      <c r="L23" s="34"/>
+      <c r="A23" s="28"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="30"/>
+      <c r="E23" s="31"/>
+      <c r="F23" s="31"/>
+      <c r="G23" s="31"/>
+      <c r="H23" s="31"/>
+      <c r="I23" s="31"/>
+      <c r="J23" s="31"/>
+      <c r="K23" s="31"/>
+      <c r="L23" s="31"/>
     </row>
     <row r="24" spans="1:12" ht="18" x14ac:dyDescent="0.3">
-      <c r="A24" s="24"/>
-      <c r="B24" s="37"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="34"/>
-      <c r="F24" s="34"/>
-      <c r="G24" s="34"/>
-      <c r="H24" s="34"/>
-      <c r="I24" s="34"/>
-      <c r="J24" s="34"/>
-      <c r="K24" s="34"/>
-      <c r="L24" s="34"/>
+      <c r="A24" s="28"/>
+      <c r="B24" s="28"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="31"/>
+      <c r="H24" s="31"/>
+      <c r="I24" s="31"/>
+      <c r="J24" s="31"/>
+      <c r="K24" s="31"/>
+      <c r="L24" s="31"/>
     </row>
     <row r="25" spans="1:12" ht="18" x14ac:dyDescent="0.3">
-      <c r="A25" s="24"/>
-      <c r="B25" s="37"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="34"/>
-      <c r="F25" s="34"/>
-      <c r="G25" s="34"/>
-      <c r="H25" s="34"/>
-      <c r="I25" s="34"/>
-      <c r="J25" s="34"/>
-      <c r="K25" s="34"/>
-      <c r="L25" s="34"/>
+      <c r="A25" s="28"/>
+      <c r="B25" s="28"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="31"/>
+      <c r="F25" s="31"/>
+      <c r="G25" s="31"/>
+      <c r="H25" s="31"/>
+      <c r="I25" s="31"/>
+      <c r="J25" s="31"/>
+      <c r="K25" s="31"/>
+      <c r="L25" s="31"/>
     </row>
     <row r="26" spans="1:12" ht="18" x14ac:dyDescent="0.3">
-      <c r="A26" s="24"/>
-      <c r="B26" s="37"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="34"/>
-      <c r="F26" s="34"/>
-      <c r="G26" s="34"/>
-      <c r="H26" s="34"/>
-      <c r="I26" s="34"/>
-      <c r="J26" s="34"/>
-      <c r="K26" s="34"/>
-      <c r="L26" s="34"/>
+      <c r="A26" s="28"/>
+      <c r="B26" s="28"/>
+      <c r="C26" s="32"/>
+      <c r="D26" s="30"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
+      <c r="L26" s="31"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A4:A6"/>
     <mergeCell ref="D4:D6"/>
@@ -1904,6 +1899,7 @@
     <mergeCell ref="G4:G6"/>
     <mergeCell ref="I4:I6"/>
     <mergeCell ref="J4:J6"/>
+    <mergeCell ref="K3:K6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>